<commit_message>
summary table for sys rev including all species
</commit_message>
<xml_diff>
--- a/data/Working_Databases/single_island_endemic_classification.xlsx
+++ b/data/Working_Databases/single_island_endemic_classification.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://connectqutedu-my.sharepoint.com/personal/n11878916_qut_edu_au/Documents/Documents/Research assistant/birds_rodents_erradication/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://connectqutedu-my.sharepoint.com/personal/n11878916_qut_edu_au/Documents/Documents/Sixth mass extinction/Luna_project/rat_evidence_review/data/Working_Databases/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="1033" documentId="8_{A10D690B-2C99-419A-9168-7ABB72A5530C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6019F2AB-AD63-4C6C-8E37-C28D162796A0}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{9080C791-29AA-4BC8-8135-E0A3210A4992}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9080C791-29AA-4BC8-8135-E0A3210A4992}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2147,11 +2147,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2167,10 +2165,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2491,15 +2485,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1429CF3-C8D8-4E78-A9A9-7DC11B99EBC4}">
   <dimension ref="A1:E341"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.81640625" customWidth="1"/>
+    <col min="1" max="1" width="40.85546875" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="21.1796875" customWidth="1"/>
-    <col min="4" max="4" width="90.453125" customWidth="1"/>
+    <col min="3" max="3" width="21.140625" customWidth="1"/>
+    <col min="4" max="4" width="90.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -2516,7 +2510,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2533,7 +2527,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -2550,7 +2544,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -2567,7 +2561,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -2584,7 +2578,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -2601,7 +2595,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -2618,7 +2612,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -2635,7 +2629,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -2652,7 +2646,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -2669,7 +2663,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -2686,7 +2680,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -2703,7 +2697,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -2720,7 +2714,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="14" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>15</v>
       </c>
@@ -2737,7 +2731,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -2754,7 +2748,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>17</v>
       </c>
@@ -2771,7 +2765,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>18</v>
       </c>
@@ -2788,7 +2782,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>19</v>
       </c>
@@ -2805,7 +2799,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>20</v>
       </c>
@@ -2822,7 +2816,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -2839,7 +2833,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>22</v>
       </c>
@@ -2856,7 +2850,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -2873,7 +2867,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>24</v>
       </c>
@@ -2890,7 +2884,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>25</v>
       </c>
@@ -2907,7 +2901,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>26</v>
       </c>
@@ -2924,7 +2918,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>27</v>
       </c>
@@ -2941,7 +2935,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>28</v>
       </c>
@@ -2958,7 +2952,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>29</v>
       </c>
@@ -2975,7 +2969,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>30</v>
       </c>
@@ -2992,7 +2986,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>31</v>
       </c>
@@ -3009,7 +3003,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>32</v>
       </c>
@@ -3026,7 +3020,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>33</v>
       </c>
@@ -3043,7 +3037,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>34</v>
       </c>
@@ -3060,7 +3054,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>35</v>
       </c>
@@ -3077,7 +3071,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>36</v>
       </c>
@@ -3094,7 +3088,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>37</v>
       </c>
@@ -3111,7 +3105,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>38</v>
       </c>
@@ -3128,7 +3122,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>39</v>
       </c>
@@ -3145,7 +3139,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>40</v>
       </c>
@@ -3162,7 +3156,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>41</v>
       </c>
@@ -3179,7 +3173,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>42</v>
       </c>
@@ -3196,7 +3190,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>43</v>
       </c>
@@ -3213,7 +3207,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>44</v>
       </c>
@@ -3230,7 +3224,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>45</v>
       </c>
@@ -3247,7 +3241,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>46</v>
       </c>
@@ -3264,7 +3258,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>47</v>
       </c>
@@ -3281,7 +3275,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>48</v>
       </c>
@@ -3298,7 +3292,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>49</v>
       </c>
@@ -3315,7 +3309,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>50</v>
       </c>
@@ -3332,7 +3326,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>51</v>
       </c>
@@ -3349,7 +3343,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>52</v>
       </c>
@@ -3366,7 +3360,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>53</v>
       </c>
@@ -3383,7 +3377,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>54</v>
       </c>
@@ -3400,7 +3394,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>55</v>
       </c>
@@ -3417,7 +3411,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>56</v>
       </c>
@@ -3434,7 +3428,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>57</v>
       </c>
@@ -3451,7 +3445,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>58</v>
       </c>
@@ -3468,7 +3462,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>59</v>
       </c>
@@ -3485,7 +3479,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>60</v>
       </c>
@@ -3502,7 +3496,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>61</v>
       </c>
@@ -3519,7 +3513,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>62</v>
       </c>
@@ -3536,7 +3530,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>63</v>
       </c>
@@ -3553,7 +3547,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>64</v>
       </c>
@@ -3570,7 +3564,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>65</v>
       </c>
@@ -3587,7 +3581,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>66</v>
       </c>
@@ -3604,7 +3598,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>67</v>
       </c>
@@ -3621,7 +3615,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>68</v>
       </c>
@@ -3638,7 +3632,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>69</v>
       </c>
@@ -3655,7 +3649,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>70</v>
       </c>
@@ -3672,7 +3666,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>71</v>
       </c>
@@ -3689,7 +3683,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>72</v>
       </c>
@@ -3706,7 +3700,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>73</v>
       </c>
@@ -3723,7 +3717,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>74</v>
       </c>
@@ -3740,7 +3734,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>75</v>
       </c>
@@ -3757,7 +3751,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>76</v>
       </c>
@@ -3774,7 +3768,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>77</v>
       </c>
@@ -3791,7 +3785,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>78</v>
       </c>
@@ -3808,7 +3802,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>79</v>
       </c>
@@ -3825,7 +3819,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>80</v>
       </c>
@@ -3842,7 +3836,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>81</v>
       </c>
@@ -3859,7 +3853,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>82</v>
       </c>
@@ -3876,7 +3870,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>83</v>
       </c>
@@ -3893,7 +3887,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>84</v>
       </c>
@@ -3910,7 +3904,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>85</v>
       </c>
@@ -3927,7 +3921,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>86</v>
       </c>
@@ -3944,7 +3938,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>87</v>
       </c>
@@ -3961,7 +3955,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>88</v>
       </c>
@@ -3978,7 +3972,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>89</v>
       </c>
@@ -3995,7 +3989,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>90</v>
       </c>
@@ -4012,7 +4006,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>91</v>
       </c>
@@ -4029,7 +4023,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>92</v>
       </c>
@@ -4046,7 +4040,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>93</v>
       </c>
@@ -4063,7 +4057,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>94</v>
       </c>
@@ -4080,7 +4074,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>95</v>
       </c>
@@ -4097,7 +4091,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>96</v>
       </c>
@@ -4114,7 +4108,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>97</v>
       </c>
@@ -4131,7 +4125,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>98</v>
       </c>
@@ -4148,7 +4142,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>99</v>
       </c>
@@ -4165,7 +4159,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>100</v>
       </c>
@@ -4182,7 +4176,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>101</v>
       </c>
@@ -4199,7 +4193,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>102</v>
       </c>
@@ -4216,7 +4210,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>103</v>
       </c>
@@ -4233,7 +4227,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>104</v>
       </c>
@@ -4250,7 +4244,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>105</v>
       </c>
@@ -4267,7 +4261,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>106</v>
       </c>
@@ -4284,7 +4278,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>107</v>
       </c>
@@ -4301,7 +4295,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>108</v>
       </c>
@@ -4318,7 +4312,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>109</v>
       </c>
@@ -4335,7 +4329,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>110</v>
       </c>
@@ -4352,7 +4346,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>111</v>
       </c>
@@ -4369,7 +4363,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>112</v>
       </c>
@@ -4386,7 +4380,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>113</v>
       </c>
@@ -4403,7 +4397,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>114</v>
       </c>
@@ -4420,7 +4414,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>115</v>
       </c>
@@ -4437,7 +4431,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>116</v>
       </c>
@@ -4454,7 +4448,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>117</v>
       </c>
@@ -4471,7 +4465,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>118</v>
       </c>
@@ -4488,7 +4482,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>119</v>
       </c>
@@ -4505,7 +4499,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>120</v>
       </c>
@@ -4522,7 +4516,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>121</v>
       </c>
@@ -4539,7 +4533,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>122</v>
       </c>
@@ -4556,7 +4550,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>123</v>
       </c>
@@ -4573,7 +4567,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>124</v>
       </c>
@@ -4590,7 +4584,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>125</v>
       </c>
@@ -4607,7 +4601,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>126</v>
       </c>
@@ -4624,7 +4618,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>127</v>
       </c>
@@ -4641,7 +4635,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>128</v>
       </c>
@@ -4658,7 +4652,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>129</v>
       </c>
@@ -4675,7 +4669,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>130</v>
       </c>
@@ -4692,7 +4686,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>131</v>
       </c>
@@ -4709,7 +4703,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>132</v>
       </c>
@@ -4726,7 +4720,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>133</v>
       </c>
@@ -4743,7 +4737,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>134</v>
       </c>
@@ -4760,7 +4754,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>135</v>
       </c>
@@ -4777,7 +4771,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>136</v>
       </c>
@@ -4794,7 +4788,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>137</v>
       </c>
@@ -4811,7 +4805,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>138</v>
       </c>
@@ -4828,7 +4822,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>139</v>
       </c>
@@ -4845,7 +4839,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>140</v>
       </c>
@@ -4862,7 +4856,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>141</v>
       </c>
@@ -4879,7 +4873,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>142</v>
       </c>
@@ -4896,7 +4890,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>143</v>
       </c>
@@ -4913,7 +4907,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>144</v>
       </c>
@@ -4930,7 +4924,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>145</v>
       </c>
@@ -4947,7 +4941,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>146</v>
       </c>
@@ -4964,7 +4958,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>147</v>
       </c>
@@ -4981,7 +4975,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>148</v>
       </c>
@@ -4998,7 +4992,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>149</v>
       </c>
@@ -5015,7 +5009,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>150</v>
       </c>
@@ -5032,7 +5026,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>151</v>
       </c>
@@ -5049,7 +5043,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>152</v>
       </c>
@@ -5066,7 +5060,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>153</v>
       </c>
@@ -5083,7 +5077,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>154</v>
       </c>
@@ -5100,7 +5094,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>155</v>
       </c>
@@ -5117,7 +5111,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>156</v>
       </c>
@@ -5134,7 +5128,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>157</v>
       </c>
@@ -5151,7 +5145,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>158</v>
       </c>
@@ -5168,7 +5162,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>159</v>
       </c>
@@ -5185,7 +5179,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>160</v>
       </c>
@@ -5202,7 +5196,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>161</v>
       </c>
@@ -5219,7 +5213,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>162</v>
       </c>
@@ -5236,7 +5230,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>163</v>
       </c>
@@ -5253,7 +5247,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>164</v>
       </c>
@@ -5270,7 +5264,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>165</v>
       </c>
@@ -5287,7 +5281,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>166</v>
       </c>
@@ -5304,7 +5298,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>167</v>
       </c>
@@ -5321,7 +5315,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>168</v>
       </c>
@@ -5338,7 +5332,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>169</v>
       </c>
@@ -5355,7 +5349,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>170</v>
       </c>
@@ -5372,7 +5366,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>171</v>
       </c>
@@ -5389,7 +5383,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>172</v>
       </c>
@@ -5406,7 +5400,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>173</v>
       </c>
@@ -5423,7 +5417,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>174</v>
       </c>
@@ -5440,7 +5434,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>175</v>
       </c>
@@ -5457,7 +5451,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>176</v>
       </c>
@@ -5474,7 +5468,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>177</v>
       </c>
@@ -5491,7 +5485,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>178</v>
       </c>
@@ -5508,7 +5502,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>179</v>
       </c>
@@ -5525,7 +5519,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>180</v>
       </c>
@@ -5542,7 +5536,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>181</v>
       </c>
@@ -5559,7 +5553,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>182</v>
       </c>
@@ -5576,7 +5570,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>183</v>
       </c>
@@ -5593,7 +5587,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>184</v>
       </c>
@@ -5610,7 +5604,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>185</v>
       </c>
@@ -5627,7 +5621,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>186</v>
       </c>
@@ -5644,7 +5638,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>187</v>
       </c>
@@ -5661,7 +5655,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>188</v>
       </c>
@@ -5678,7 +5672,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>189</v>
       </c>
@@ -5695,7 +5689,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>190</v>
       </c>
@@ -5712,7 +5706,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>191</v>
       </c>
@@ -5729,7 +5723,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>192</v>
       </c>
@@ -5746,7 +5740,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>193</v>
       </c>
@@ -5763,7 +5757,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>194</v>
       </c>
@@ -5780,7 +5774,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>195</v>
       </c>
@@ -5797,7 +5791,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>196</v>
       </c>
@@ -5814,7 +5808,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="196" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A196" s="1" t="s">
         <v>197</v>
       </c>
@@ -5831,7 +5825,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>198</v>
       </c>
@@ -5848,7 +5842,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>199</v>
       </c>
@@ -5865,7 +5859,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>200</v>
       </c>
@@ -5882,7 +5876,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>201</v>
       </c>
@@ -5899,7 +5893,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>202</v>
       </c>
@@ -5916,7 +5910,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>203</v>
       </c>
@@ -5933,7 +5927,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>204</v>
       </c>
@@ -5950,7 +5944,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>205</v>
       </c>
@@ -5967,7 +5961,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>206</v>
       </c>
@@ -5984,7 +5978,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>207</v>
       </c>
@@ -6001,7 +5995,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>208</v>
       </c>
@@ -6018,7 +6012,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="208" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A208" s="1" t="s">
         <v>209</v>
       </c>
@@ -6035,7 +6029,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>210</v>
       </c>
@@ -6052,7 +6046,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
         <v>211</v>
       </c>
@@ -6069,7 +6063,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
         <v>212</v>
       </c>
@@ -6086,7 +6080,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
         <v>213</v>
       </c>
@@ -6103,7 +6097,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
         <v>214</v>
       </c>
@@ -6120,7 +6114,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
         <v>215</v>
       </c>
@@ -6137,7 +6131,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>216</v>
       </c>
@@ -6154,7 +6148,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
         <v>217</v>
       </c>
@@ -6171,7 +6165,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
         <v>218</v>
       </c>
@@ -6188,7 +6182,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
         <v>219</v>
       </c>
@@ -6205,7 +6199,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
         <v>220</v>
       </c>
@@ -6222,7 +6216,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
         <v>221</v>
       </c>
@@ -6239,7 +6233,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>222</v>
       </c>
@@ -6256,7 +6250,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
         <v>223</v>
       </c>
@@ -6273,7 +6267,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
         <v>224</v>
       </c>
@@ -6290,7 +6284,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>225</v>
       </c>
@@ -6307,7 +6301,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>226</v>
       </c>
@@ -6324,7 +6318,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>227</v>
       </c>
@@ -6341,7 +6335,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>228</v>
       </c>
@@ -6358,7 +6352,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
         <v>229</v>
       </c>
@@ -6375,7 +6369,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
         <v>230</v>
       </c>
@@ -6392,7 +6386,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
         <v>231</v>
       </c>
@@ -6409,7 +6403,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>232</v>
       </c>
@@ -6426,7 +6420,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
         <v>233</v>
       </c>
@@ -6443,7 +6437,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>234</v>
       </c>
@@ -6460,7 +6454,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
         <v>235</v>
       </c>
@@ -6477,7 +6471,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>236</v>
       </c>
@@ -6494,7 +6488,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
         <v>237</v>
       </c>
@@ -6511,7 +6505,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
         <v>238</v>
       </c>
@@ -6528,7 +6522,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
         <v>239</v>
       </c>
@@ -6545,7 +6539,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
         <v>240</v>
       </c>
@@ -6562,7 +6556,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
         <v>241</v>
       </c>
@@ -6579,7 +6573,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
         <v>242</v>
       </c>
@@ -6596,7 +6590,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
         <v>243</v>
       </c>
@@ -6613,7 +6607,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
         <v>244</v>
       </c>
@@ -6630,7 +6624,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
         <v>245</v>
       </c>
@@ -6647,7 +6641,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
         <v>246</v>
       </c>
@@ -6664,7 +6658,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
         <v>247</v>
       </c>
@@ -6681,7 +6675,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="247" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
         <v>248</v>
       </c>
@@ -6698,7 +6692,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="248" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
         <v>249</v>
       </c>
@@ -6715,7 +6709,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="249" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
         <v>250</v>
       </c>
@@ -6732,7 +6726,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="250" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
         <v>251</v>
       </c>
@@ -6749,7 +6743,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="251" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
         <v>252</v>
       </c>
@@ -6766,7 +6760,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="252" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
         <v>253</v>
       </c>
@@ -6783,7 +6777,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="253" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
         <v>254</v>
       </c>
@@ -6800,7 +6794,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="254" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
         <v>255</v>
       </c>
@@ -6817,7 +6811,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="255" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
         <v>256</v>
       </c>
@@ -6827,14 +6821,14 @@
       <c r="C255" t="s">
         <v>344</v>
       </c>
-      <c r="D255" s="2" t="s">
+      <c r="D255" t="s">
         <v>600</v>
       </c>
       <c r="E255" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="256" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
         <v>257</v>
       </c>
@@ -6844,14 +6838,14 @@
       <c r="C256" t="s">
         <v>349</v>
       </c>
-      <c r="D256" s="2" t="s">
+      <c r="D256" t="s">
         <v>601</v>
       </c>
       <c r="E256" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="257" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
         <v>258</v>
       </c>
@@ -6861,14 +6855,14 @@
       <c r="C257" t="s">
         <v>344</v>
       </c>
-      <c r="D257" s="2" t="s">
+      <c r="D257" t="s">
         <v>602</v>
       </c>
       <c r="E257" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="258" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
         <v>259</v>
       </c>
@@ -6878,14 +6872,14 @@
       <c r="C258" t="s">
         <v>344</v>
       </c>
-      <c r="D258" s="2" t="s">
+      <c r="D258" t="s">
         <v>603</v>
       </c>
       <c r="E258" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="259" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
         <v>260</v>
       </c>
@@ -6895,14 +6889,14 @@
       <c r="C259" t="s">
         <v>344</v>
       </c>
-      <c r="D259" s="2" t="s">
+      <c r="D259" t="s">
         <v>604</v>
       </c>
       <c r="E259" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="260" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
         <v>261</v>
       </c>
@@ -6912,14 +6906,14 @@
       <c r="C260" t="s">
         <v>344</v>
       </c>
-      <c r="D260" s="2" t="s">
+      <c r="D260" t="s">
         <v>605</v>
       </c>
       <c r="E260" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="261" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
         <v>262</v>
       </c>
@@ -6929,14 +6923,14 @@
       <c r="C261" t="s">
         <v>344</v>
       </c>
-      <c r="D261" s="2" t="s">
+      <c r="D261" t="s">
         <v>606</v>
       </c>
       <c r="E261" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="262" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
         <v>263</v>
       </c>
@@ -6946,14 +6940,14 @@
       <c r="C262" t="s">
         <v>344</v>
       </c>
-      <c r="D262" s="2" t="s">
+      <c r="D262" t="s">
         <v>607</v>
       </c>
       <c r="E262" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="263" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
         <v>264</v>
       </c>
@@ -6963,14 +6957,14 @@
       <c r="C263" t="s">
         <v>344</v>
       </c>
-      <c r="D263" s="2" t="s">
+      <c r="D263" t="s">
         <v>608</v>
       </c>
       <c r="E263" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
         <v>265</v>
       </c>
@@ -6980,14 +6974,14 @@
       <c r="C264" t="s">
         <v>344</v>
       </c>
-      <c r="D264" s="2" t="s">
+      <c r="D264" t="s">
         <v>609</v>
       </c>
       <c r="E264" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="265" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
         <v>266</v>
       </c>
@@ -6997,14 +6991,14 @@
       <c r="C265" t="s">
         <v>344</v>
       </c>
-      <c r="D265" s="2" t="s">
+      <c r="D265" t="s">
         <v>610</v>
       </c>
       <c r="E265" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="266" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
         <v>267</v>
       </c>
@@ -7014,14 +7008,14 @@
       <c r="C266" t="s">
         <v>344</v>
       </c>
-      <c r="D266" s="2" t="s">
+      <c r="D266" t="s">
         <v>611</v>
       </c>
       <c r="E266" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="267" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
         <v>268</v>
       </c>
@@ -7031,14 +7025,14 @@
       <c r="C267" t="s">
         <v>344</v>
       </c>
-      <c r="D267" s="2" t="s">
+      <c r="D267" t="s">
         <v>612</v>
       </c>
       <c r="E267" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="268" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
         <v>269</v>
       </c>
@@ -7048,14 +7042,14 @@
       <c r="C268" t="s">
         <v>344</v>
       </c>
-      <c r="D268" s="2" t="s">
+      <c r="D268" t="s">
         <v>613</v>
       </c>
       <c r="E268" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="269" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
         <v>270</v>
       </c>
@@ -7065,14 +7059,14 @@
       <c r="C269" t="s">
         <v>344</v>
       </c>
-      <c r="D269" s="2" t="s">
+      <c r="D269" t="s">
         <v>614</v>
       </c>
       <c r="E269" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
         <v>271</v>
       </c>
@@ -7082,14 +7076,14 @@
       <c r="C270" t="s">
         <v>344</v>
       </c>
-      <c r="D270" s="2" t="s">
+      <c r="D270" t="s">
         <v>615</v>
       </c>
       <c r="E270" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
         <v>272</v>
       </c>
@@ -7099,14 +7093,14 @@
       <c r="C271" t="s">
         <v>344</v>
       </c>
-      <c r="D271" s="2" t="s">
+      <c r="D271" t="s">
         <v>616</v>
       </c>
       <c r="E271" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="272" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
         <v>273</v>
       </c>
@@ -7116,14 +7110,14 @@
       <c r="C272" t="s">
         <v>344</v>
       </c>
-      <c r="D272" s="2" t="s">
+      <c r="D272" t="s">
         <v>617</v>
       </c>
       <c r="E272" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="273" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
         <v>274</v>
       </c>
@@ -7133,14 +7127,14 @@
       <c r="C273" t="s">
         <v>349</v>
       </c>
-      <c r="D273" s="2" t="s">
+      <c r="D273" t="s">
         <v>618</v>
       </c>
       <c r="E273" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="274" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
         <v>275</v>
       </c>
@@ -7150,14 +7144,14 @@
       <c r="C274" t="s">
         <v>344</v>
       </c>
-      <c r="D274" s="2" t="s">
+      <c r="D274" t="s">
         <v>619</v>
       </c>
       <c r="E274" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="275" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
         <v>276</v>
       </c>
@@ -7167,14 +7161,14 @@
       <c r="C275" t="s">
         <v>344</v>
       </c>
-      <c r="D275" s="2" t="s">
+      <c r="D275" t="s">
         <v>620</v>
       </c>
       <c r="E275" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="276" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
         <v>277</v>
       </c>
@@ -7184,14 +7178,14 @@
       <c r="C276" t="s">
         <v>344</v>
       </c>
-      <c r="D276" s="2" t="s">
+      <c r="D276" t="s">
         <v>621</v>
       </c>
       <c r="E276" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="277" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
         <v>278</v>
       </c>
@@ -7201,14 +7195,14 @@
       <c r="C277" t="s">
         <v>344</v>
       </c>
-      <c r="D277" s="2" t="s">
+      <c r="D277" t="s">
         <v>622</v>
       </c>
       <c r="E277" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="278" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
         <v>279</v>
       </c>
@@ -7218,14 +7212,14 @@
       <c r="C278" t="s">
         <v>344</v>
       </c>
-      <c r="D278" s="2" t="s">
+      <c r="D278" t="s">
         <v>623</v>
       </c>
       <c r="E278" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="279" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
         <v>280</v>
       </c>
@@ -7235,14 +7229,14 @@
       <c r="C279" t="s">
         <v>344</v>
       </c>
-      <c r="D279" s="2" t="s">
+      <c r="D279" t="s">
         <v>624</v>
       </c>
       <c r="E279" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="280" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
         <v>281</v>
       </c>
@@ -7252,14 +7246,14 @@
       <c r="C280" t="s">
         <v>344</v>
       </c>
-      <c r="D280" s="2" t="s">
+      <c r="D280" t="s">
         <v>625</v>
       </c>
       <c r="E280" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="281" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
         <v>282</v>
       </c>
@@ -7269,14 +7263,14 @@
       <c r="C281" t="s">
         <v>344</v>
       </c>
-      <c r="D281" s="2" t="s">
+      <c r="D281" t="s">
         <v>626</v>
       </c>
       <c r="E281" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="282" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
         <v>283</v>
       </c>
@@ -7286,14 +7280,14 @@
       <c r="C282" t="s">
         <v>344</v>
       </c>
-      <c r="D282" s="2" t="s">
+      <c r="D282" t="s">
         <v>627</v>
       </c>
       <c r="E282" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="283" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
         <v>284</v>
       </c>
@@ -7303,14 +7297,14 @@
       <c r="C283" t="s">
         <v>344</v>
       </c>
-      <c r="D283" s="2" t="s">
+      <c r="D283" t="s">
         <v>628</v>
       </c>
       <c r="E283" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="284" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
         <v>285</v>
       </c>
@@ -7320,14 +7314,14 @@
       <c r="C284" t="s">
         <v>344</v>
       </c>
-      <c r="D284" s="2" t="s">
+      <c r="D284" t="s">
         <v>629</v>
       </c>
       <c r="E284" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="285" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
         <v>286</v>
       </c>
@@ -7337,14 +7331,14 @@
       <c r="C285" t="s">
         <v>349</v>
       </c>
-      <c r="D285" s="2" t="s">
+      <c r="D285" t="s">
         <v>631</v>
       </c>
       <c r="E285" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="286" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
         <v>287</v>
       </c>
@@ -7354,14 +7348,14 @@
       <c r="C286" t="s">
         <v>344</v>
       </c>
-      <c r="D286" s="2" t="s">
+      <c r="D286" t="s">
         <v>630</v>
       </c>
       <c r="E286" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="287" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
         <v>288</v>
       </c>
@@ -7371,14 +7365,14 @@
       <c r="C287" t="s">
         <v>344</v>
       </c>
-      <c r="D287" s="2" t="s">
+      <c r="D287" t="s">
         <v>632</v>
       </c>
       <c r="E287" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="288" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
         <v>289</v>
       </c>
@@ -7388,14 +7382,14 @@
       <c r="C288" t="s">
         <v>344</v>
       </c>
-      <c r="D288" s="2" t="s">
+      <c r="D288" t="s">
         <v>633</v>
       </c>
       <c r="E288" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="289" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
         <v>290</v>
       </c>
@@ -7405,14 +7399,14 @@
       <c r="C289" t="s">
         <v>344</v>
       </c>
-      <c r="D289" s="2" t="s">
+      <c r="D289" t="s">
         <v>634</v>
       </c>
       <c r="E289" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="290" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
         <v>291</v>
       </c>
@@ -7422,14 +7416,14 @@
       <c r="C290" t="s">
         <v>349</v>
       </c>
-      <c r="D290" s="2" t="s">
+      <c r="D290" t="s">
         <v>635</v>
       </c>
       <c r="E290" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="291" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
         <v>292</v>
       </c>
@@ -7439,14 +7433,14 @@
       <c r="C291" t="s">
         <v>344</v>
       </c>
-      <c r="D291" s="2" t="s">
+      <c r="D291" t="s">
         <v>636</v>
       </c>
       <c r="E291" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="292" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A292" s="1" t="s">
         <v>293</v>
       </c>
@@ -7456,14 +7450,14 @@
       <c r="C292" s="1" t="s">
         <v>349</v>
       </c>
-      <c r="D292" s="3" t="s">
+      <c r="D292" s="1" t="s">
         <v>637</v>
       </c>
       <c r="E292" s="1" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="293" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
         <v>294</v>
       </c>
@@ -7473,14 +7467,14 @@
       <c r="C293" t="s">
         <v>344</v>
       </c>
-      <c r="D293" s="2" t="s">
+      <c r="D293" t="s">
         <v>638</v>
       </c>
       <c r="E293" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="294" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
         <v>295</v>
       </c>
@@ -7490,14 +7484,14 @@
       <c r="C294" t="s">
         <v>349</v>
       </c>
-      <c r="D294" s="2" t="s">
+      <c r="D294" t="s">
         <v>639</v>
       </c>
       <c r="E294" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="295" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
         <v>296</v>
       </c>
@@ -7507,14 +7501,14 @@
       <c r="C295" t="s">
         <v>344</v>
       </c>
-      <c r="D295" s="2" t="s">
+      <c r="D295" t="s">
         <v>640</v>
       </c>
       <c r="E295" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="296" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
         <v>297</v>
       </c>
@@ -7524,14 +7518,14 @@
       <c r="C296" t="s">
         <v>344</v>
       </c>
-      <c r="D296" s="2" t="s">
+      <c r="D296" t="s">
         <v>641</v>
       </c>
       <c r="E296" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="297" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
         <v>298</v>
       </c>
@@ -7541,14 +7535,14 @@
       <c r="C297" t="s">
         <v>344</v>
       </c>
-      <c r="D297" s="2" t="s">
+      <c r="D297" t="s">
         <v>642</v>
       </c>
       <c r="E297" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="298" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
         <v>299</v>
       </c>
@@ -7558,14 +7552,14 @@
       <c r="C298" t="s">
         <v>344</v>
       </c>
-      <c r="D298" s="2" t="s">
+      <c r="D298" t="s">
         <v>643</v>
       </c>
       <c r="E298" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="299" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
         <v>300</v>
       </c>
@@ -7575,14 +7569,14 @@
       <c r="C299" t="s">
         <v>344</v>
       </c>
-      <c r="D299" s="2" t="s">
+      <c r="D299" t="s">
         <v>644</v>
       </c>
       <c r="E299" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="300" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
         <v>301</v>
       </c>
@@ -7592,14 +7586,14 @@
       <c r="C300" t="s">
         <v>344</v>
       </c>
-      <c r="D300" s="2" t="s">
+      <c r="D300" t="s">
         <v>645</v>
       </c>
       <c r="E300" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="301" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
         <v>302</v>
       </c>
@@ -7609,14 +7603,14 @@
       <c r="C301" t="s">
         <v>344</v>
       </c>
-      <c r="D301" s="2" t="s">
+      <c r="D301" t="s">
         <v>646</v>
       </c>
       <c r="E301" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="302" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
         <v>303</v>
       </c>
@@ -7626,14 +7620,14 @@
       <c r="C302" t="s">
         <v>344</v>
       </c>
-      <c r="D302" s="2" t="s">
+      <c r="D302" t="s">
         <v>647</v>
       </c>
       <c r="E302" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="303" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
         <v>304</v>
       </c>
@@ -7643,14 +7637,14 @@
       <c r="C303" t="s">
         <v>344</v>
       </c>
-      <c r="D303" s="2" t="s">
+      <c r="D303" t="s">
         <v>648</v>
       </c>
       <c r="E303" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="304" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
         <v>305</v>
       </c>
@@ -7660,14 +7654,14 @@
       <c r="C304" t="s">
         <v>344</v>
       </c>
-      <c r="D304" s="2" t="s">
+      <c r="D304" t="s">
         <v>649</v>
       </c>
       <c r="E304" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="305" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
         <v>306</v>
       </c>
@@ -7677,14 +7671,14 @@
       <c r="C305" t="s">
         <v>349</v>
       </c>
-      <c r="D305" s="2" t="s">
+      <c r="D305" t="s">
         <v>650</v>
       </c>
       <c r="E305" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="306" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
         <v>307</v>
       </c>
@@ -7694,14 +7688,14 @@
       <c r="C306" t="s">
         <v>344</v>
       </c>
-      <c r="D306" s="2" t="s">
+      <c r="D306" t="s">
         <v>651</v>
       </c>
       <c r="E306" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="307" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
         <v>308</v>
       </c>
@@ -7711,14 +7705,14 @@
       <c r="C307" t="s">
         <v>344</v>
       </c>
-      <c r="D307" s="2" t="s">
+      <c r="D307" t="s">
         <v>652</v>
       </c>
       <c r="E307" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="308" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
         <v>309</v>
       </c>
@@ -7728,14 +7722,14 @@
       <c r="C308" t="s">
         <v>344</v>
       </c>
-      <c r="D308" s="2" t="s">
+      <c r="D308" t="s">
         <v>653</v>
       </c>
       <c r="E308" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="309" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
         <v>310</v>
       </c>
@@ -7745,14 +7739,14 @@
       <c r="C309" t="s">
         <v>344</v>
       </c>
-      <c r="D309" s="2" t="s">
+      <c r="D309" t="s">
         <v>654</v>
       </c>
       <c r="E309" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="310" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
         <v>311</v>
       </c>
@@ -7762,14 +7756,14 @@
       <c r="C310" t="s">
         <v>344</v>
       </c>
-      <c r="D310" s="2" t="s">
+      <c r="D310" t="s">
         <v>655</v>
       </c>
       <c r="E310" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="311" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
         <v>312</v>
       </c>
@@ -7779,14 +7773,14 @@
       <c r="C311" t="s">
         <v>349</v>
       </c>
-      <c r="D311" s="2" t="s">
+      <c r="D311" t="s">
         <v>656</v>
       </c>
       <c r="E311" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="312" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
         <v>313</v>
       </c>
@@ -7796,14 +7790,14 @@
       <c r="C312" t="s">
         <v>344</v>
       </c>
-      <c r="D312" s="2" t="s">
+      <c r="D312" t="s">
         <v>657</v>
       </c>
       <c r="E312" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="313" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
         <v>314</v>
       </c>
@@ -7813,14 +7807,14 @@
       <c r="C313" t="s">
         <v>344</v>
       </c>
-      <c r="D313" s="2" t="s">
+      <c r="D313" t="s">
         <v>658</v>
       </c>
       <c r="E313" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="314" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
         <v>315</v>
       </c>
@@ -7830,14 +7824,14 @@
       <c r="C314" t="s">
         <v>344</v>
       </c>
-      <c r="D314" s="2" t="s">
+      <c r="D314" t="s">
         <v>659</v>
       </c>
       <c r="E314" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="315" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A315" s="1" t="s">
         <v>316</v>
       </c>
@@ -7847,14 +7841,14 @@
       <c r="C315" s="1" t="s">
         <v>344</v>
       </c>
-      <c r="D315" s="3" t="s">
+      <c r="D315" s="1" t="s">
         <v>660</v>
       </c>
       <c r="E315" s="1" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="316" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
         <v>317</v>
       </c>
@@ -7864,14 +7858,14 @@
       <c r="C316" t="s">
         <v>344</v>
       </c>
-      <c r="D316" s="2" t="s">
+      <c r="D316" t="s">
         <v>661</v>
       </c>
       <c r="E316" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="317" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
         <v>318</v>
       </c>
@@ -7881,14 +7875,14 @@
       <c r="C317" t="s">
         <v>344</v>
       </c>
-      <c r="D317" s="2" t="s">
+      <c r="D317" t="s">
         <v>662</v>
       </c>
       <c r="E317" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="318" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
         <v>319</v>
       </c>
@@ -7898,14 +7892,14 @@
       <c r="C318" t="s">
         <v>349</v>
       </c>
-      <c r="D318" s="2" t="s">
+      <c r="D318" t="s">
         <v>663</v>
       </c>
       <c r="E318" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="319" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
         <v>320</v>
       </c>
@@ -7915,14 +7909,14 @@
       <c r="C319" t="s">
         <v>349</v>
       </c>
-      <c r="D319" s="2" t="s">
+      <c r="D319" t="s">
         <v>664</v>
       </c>
       <c r="E319" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="320" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
         <v>321</v>
       </c>
@@ -7932,14 +7926,14 @@
       <c r="C320" t="s">
         <v>349</v>
       </c>
-      <c r="D320" s="2" t="s">
+      <c r="D320" t="s">
         <v>665</v>
       </c>
       <c r="E320" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="321" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
         <v>322</v>
       </c>
@@ -7949,14 +7943,14 @@
       <c r="C321" t="s">
         <v>349</v>
       </c>
-      <c r="D321" s="2" t="s">
+      <c r="D321" t="s">
         <v>666</v>
       </c>
       <c r="E321" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="322" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
         <v>323</v>
       </c>
@@ -7966,14 +7960,14 @@
       <c r="C322" t="s">
         <v>344</v>
       </c>
-      <c r="D322" s="2" t="s">
+      <c r="D322" t="s">
         <v>667</v>
       </c>
       <c r="E322" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="323" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
         <v>324</v>
       </c>
@@ -7983,14 +7977,14 @@
       <c r="C323" t="s">
         <v>344</v>
       </c>
-      <c r="D323" s="2" t="s">
+      <c r="D323" t="s">
         <v>668</v>
       </c>
       <c r="E323" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="324" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A324" s="1" t="s">
         <v>325</v>
       </c>
@@ -8000,14 +7994,14 @@
       <c r="C324" s="1" t="s">
         <v>344</v>
       </c>
-      <c r="D324" s="3" t="s">
+      <c r="D324" s="1" t="s">
         <v>669</v>
       </c>
       <c r="E324" s="1" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="325" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
         <v>326</v>
       </c>
@@ -8017,14 +8011,14 @@
       <c r="C325" t="s">
         <v>349</v>
       </c>
-      <c r="D325" s="2" t="s">
+      <c r="D325" t="s">
         <v>670</v>
       </c>
       <c r="E325" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="326" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
         <v>327</v>
       </c>
@@ -8034,14 +8028,14 @@
       <c r="C326" t="s">
         <v>349</v>
       </c>
-      <c r="D326" s="2" t="s">
+      <c r="D326" t="s">
         <v>382</v>
       </c>
       <c r="E326" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="327" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
         <v>328</v>
       </c>
@@ -8051,14 +8045,14 @@
       <c r="C327" t="s">
         <v>344</v>
       </c>
-      <c r="D327" s="2" t="s">
+      <c r="D327" t="s">
         <v>671</v>
       </c>
       <c r="E327" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="328" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
         <v>329</v>
       </c>
@@ -8068,14 +8062,14 @@
       <c r="C328" t="s">
         <v>349</v>
       </c>
-      <c r="D328" s="2" t="s">
+      <c r="D328" t="s">
         <v>672</v>
       </c>
       <c r="E328" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="329" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A329" t="s">
         <v>330</v>
       </c>
@@ -8085,14 +8079,14 @@
       <c r="C329" t="s">
         <v>349</v>
       </c>
-      <c r="D329" s="2" t="s">
+      <c r="D329" t="s">
         <v>673</v>
       </c>
       <c r="E329" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="330" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
         <v>331</v>
       </c>
@@ -8102,14 +8096,14 @@
       <c r="C330" t="s">
         <v>349</v>
       </c>
-      <c r="D330" s="2" t="s">
+      <c r="D330" t="s">
         <v>674</v>
       </c>
       <c r="E330" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="331" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
         <v>332</v>
       </c>
@@ -8119,14 +8113,14 @@
       <c r="C331" t="s">
         <v>349</v>
       </c>
-      <c r="D331" s="2" t="s">
+      <c r="D331" t="s">
         <v>675</v>
       </c>
       <c r="E331" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="332" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
         <v>333</v>
       </c>
@@ -8136,14 +8130,14 @@
       <c r="C332" t="s">
         <v>349</v>
       </c>
-      <c r="D332" s="2" t="s">
+      <c r="D332" t="s">
         <v>676</v>
       </c>
       <c r="E332" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="333" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
         <v>334</v>
       </c>
@@ -8153,14 +8147,14 @@
       <c r="C333" t="s">
         <v>349</v>
       </c>
-      <c r="D333" s="2" t="s">
+      <c r="D333" t="s">
         <v>677</v>
       </c>
       <c r="E333" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="334" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
         <v>335</v>
       </c>
@@ -8170,14 +8164,14 @@
       <c r="C334" t="s">
         <v>349</v>
       </c>
-      <c r="D334" s="2" t="s">
+      <c r="D334" t="s">
         <v>678</v>
       </c>
       <c r="E334" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="335" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
         <v>336</v>
       </c>
@@ -8187,14 +8181,14 @@
       <c r="C335" t="s">
         <v>349</v>
       </c>
-      <c r="D335" s="2" t="s">
+      <c r="D335" t="s">
         <v>679</v>
       </c>
       <c r="E335" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="336" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A336" t="s">
         <v>337</v>
       </c>
@@ -8204,14 +8198,14 @@
       <c r="C336" t="s">
         <v>344</v>
       </c>
-      <c r="D336" s="2" t="s">
+      <c r="D336" t="s">
         <v>680</v>
       </c>
       <c r="E336" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="337" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A337" t="s">
         <v>338</v>
       </c>
@@ -8221,14 +8215,14 @@
       <c r="C337" t="s">
         <v>349</v>
       </c>
-      <c r="D337" s="2" t="s">
+      <c r="D337" t="s">
         <v>681</v>
       </c>
       <c r="E337" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="338" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
         <v>339</v>
       </c>
@@ -8238,14 +8232,14 @@
       <c r="C338" t="s">
         <v>349</v>
       </c>
-      <c r="D338" s="2" t="s">
+      <c r="D338" t="s">
         <v>682</v>
       </c>
       <c r="E338" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="339" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
         <v>340</v>
       </c>
@@ -8255,14 +8249,14 @@
       <c r="C339" t="s">
         <v>349</v>
       </c>
-      <c r="D339" s="2" t="s">
+      <c r="D339" t="s">
         <v>683</v>
       </c>
       <c r="E339" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="340" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
         <v>341</v>
       </c>
@@ -8272,14 +8266,14 @@
       <c r="C340" t="s">
         <v>349</v>
       </c>
-      <c r="D340" s="2" t="s">
+      <c r="D340" t="s">
         <v>684</v>
       </c>
       <c r="E340" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="341" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
         <v>342</v>
       </c>
@@ -8289,7 +8283,7 @@
       <c r="C341" t="s">
         <v>349</v>
       </c>
-      <c r="D341" s="2" t="s">
+      <c r="D341" t="s">
         <v>685</v>
       </c>
       <c r="E341" t="s">

</xml_diff>